<commit_message>
Add network notes column to customer tracker
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNKQUt1mvoZR5vMj2W2kRm
</commit_message>
<xml_diff>
--- a/customer-tracker/onehome_customer_tracker_SAMPLE.xlsx
+++ b/customer-tracker/onehome_customer_tracker_SAMPLE.xlsx
@@ -128,7 +128,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Z1" authorId="0">
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -217,7 +217,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="AE1" authorId="0">
+    <comment ref="AF1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -274,7 +274,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="AF1" authorId="0">
+    <comment ref="AG1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -331,7 +331,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="AG1" authorId="0">
+    <comment ref="AH1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -543,7 +543,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="165">
   <si>
     <t xml:space="preserve">OneHome — גיליון מעקב לקוחות (קובץ דוגמה)</t>
   </si>
@@ -599,6 +599,9 @@
     <t xml:space="preserve">7. בדיקת ה-SLA מניחה ימי עסקים א׳–ה׳ בלי חגים, והיעד הוא סוף יום העסקים ה-N אחרי פתיחת הפנייה. אם שישי נחשב יום עסקים, לתקן את הנוסחה בעמודה "יעד SLA".</t>
   </si>
   <si>
+    <t xml:space="preserve">8. "הערות רשת" — רושמים רק חריגות ממוסכמת הסיומות (HA ב-50, Shelly ב-60 עד 79 וכו' — ראו plan-site/kb.html), למשל "50 תפוסה, ה-HA ב-51" או "הראוטר לא מאפשר reservation". אם אין חריגה, כותבים "—".</t>
+  </si>
+  <si>
     <t xml:space="preserve">מזהה לקוח</t>
   </si>
   <si>
@@ -662,6 +665,9 @@
     <t xml:space="preserve">MAC של ה-HA</t>
   </si>
   <si>
+    <t xml:space="preserve">הערות רשת (חריגות IP)</t>
+  </si>
+  <si>
     <t xml:space="preserve">גרסת HA</t>
   </si>
   <si>
@@ -737,13 +743,13 @@
     <t xml:space="preserve">AA:BB:CC:DD:EE:FF</t>
   </si>
   <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026.9.3</t>
   </si>
   <si>
     <t xml:space="preserve">לא</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">onehome-c001-backups</t>
@@ -1612,7 +1618,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1715,6 +1721,11 @@
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1733,7 +1744,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AL21"/>
+  <dimension ref="A1:AM21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1751,153 +1762,157 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="34" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="37" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="25" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="35" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="38" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Z1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AA1" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AC1" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AE1" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AF1" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AH1" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AI1" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AJ1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AK1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AL1" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F2" s="6" t="n">
         <f aca="false">IF($E2="","",IFERROR(INDEX(חבילות!$B$2:$B$4,MATCH($E2,חבילות!$A$2:$A$4,0)),""))</f>
@@ -1946,70 +1961,73 @@
         <v>46314</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="X2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="Z2" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AB2" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="AC2" s="7" t="n">
+        <v>71</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="AD2" s="7" t="n">
         <v>4200</v>
       </c>
-      <c r="AD2" s="7" t="n">
+      <c r="AE2" s="7" t="n">
         <v>800</v>
       </c>
-      <c r="AE2" s="11" t="n">
-        <f aca="false">IF(OR($A2="",$I2="",$AC2=""),"",$I2-$AC2-N($AD2))</f>
+      <c r="AF2" s="11" t="n">
+        <f aca="false">IF(OR($A2="",$I2="",$AD2=""),"",$I2-$AD2-N($AE2))</f>
         <v>3700</v>
       </c>
-      <c r="AF2" s="12" t="n">
+      <c r="AG2" s="12" t="n">
         <f aca="false">IF($A2="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A2,Checklist!$C$1:$G$1,0)),""))</f>
         <v>1</v>
       </c>
-      <c r="AG2" s="13" t="n">
+      <c r="AH2" s="13" t="n">
         <f aca="false">IF($A2="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A2)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A2,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v>18.5</v>
       </c>
-      <c r="AH2" s="11" t="n">
-        <f aca="false">IF($A2="","",IFERROR($AE2/$AG2,""))</f>
+      <c r="AI2" s="11" t="n">
+        <f aca="false">IF($A2="","",IFERROR($AF2/$AH2,""))</f>
         <v>200</v>
       </c>
-      <c r="AI2" s="13" t="n">
+      <c r="AJ2" s="13" t="n">
         <f aca="false">IF($A2="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A2,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v>1.5</v>
       </c>
-      <c r="AJ2" s="9" t="n">
+      <c r="AK2" s="9" t="n">
         <f aca="false">IF($A2="","",COUNTIFS(פניות!$B$2:$B$500,$A2,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v>1</v>
       </c>
-      <c r="AK2" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="AL2" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2062,34 +2080,35 @@
       <c r="Z3" s="5"/>
       <c r="AA3" s="5"/>
       <c r="AB3" s="5"/>
-      <c r="AC3" s="7"/>
+      <c r="AC3" s="5"/>
       <c r="AD3" s="7"/>
-      <c r="AE3" s="11" t="str">
-        <f aca="false">IF(OR($A3="",$I3="",$AC3=""),"",$I3-$AC3-N($AD3))</f>
-        <v/>
-      </c>
-      <c r="AF3" s="12" t="str">
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="11" t="str">
+        <f aca="false">IF(OR($A3="",$I3="",$AD3=""),"",$I3-$AD3-N($AE3))</f>
+        <v/>
+      </c>
+      <c r="AG3" s="12" t="str">
         <f aca="false">IF($A3="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A3,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG3" s="13" t="str">
+      <c r="AH3" s="13" t="str">
         <f aca="false">IF($A3="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A3)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A3,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH3" s="11" t="str">
-        <f aca="false">IF($A3="","",IFERROR($AE3/$AG3,""))</f>
-        <v/>
-      </c>
-      <c r="AI3" s="13" t="str">
+      <c r="AI3" s="11" t="str">
+        <f aca="false">IF($A3="","",IFERROR($AF3/$AH3,""))</f>
+        <v/>
+      </c>
+      <c r="AJ3" s="13" t="str">
         <f aca="false">IF($A3="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A3,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ3" s="9" t="str">
+      <c r="AK3" s="9" t="str">
         <f aca="false">IF($A3="","",COUNTIFS(פניות!$B$2:$B$500,$A3,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK3" s="5"/>
       <c r="AL3" s="5"/>
+      <c r="AM3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5"/>
@@ -2141,34 +2160,35 @@
       <c r="Z4" s="5"/>
       <c r="AA4" s="5"/>
       <c r="AB4" s="5"/>
-      <c r="AC4" s="7"/>
+      <c r="AC4" s="5"/>
       <c r="AD4" s="7"/>
-      <c r="AE4" s="11" t="str">
-        <f aca="false">IF(OR($A4="",$I4="",$AC4=""),"",$I4-$AC4-N($AD4))</f>
-        <v/>
-      </c>
-      <c r="AF4" s="12" t="str">
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="11" t="str">
+        <f aca="false">IF(OR($A4="",$I4="",$AD4=""),"",$I4-$AD4-N($AE4))</f>
+        <v/>
+      </c>
+      <c r="AG4" s="12" t="str">
         <f aca="false">IF($A4="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A4,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG4" s="13" t="str">
+      <c r="AH4" s="13" t="str">
         <f aca="false">IF($A4="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A4)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A4,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH4" s="11" t="str">
-        <f aca="false">IF($A4="","",IFERROR($AE4/$AG4,""))</f>
-        <v/>
-      </c>
-      <c r="AI4" s="13" t="str">
+      <c r="AI4" s="11" t="str">
+        <f aca="false">IF($A4="","",IFERROR($AF4/$AH4,""))</f>
+        <v/>
+      </c>
+      <c r="AJ4" s="13" t="str">
         <f aca="false">IF($A4="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A4,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ4" s="9" t="str">
+      <c r="AK4" s="9" t="str">
         <f aca="false">IF($A4="","",COUNTIFS(פניות!$B$2:$B$500,$A4,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK4" s="5"/>
       <c r="AL4" s="5"/>
+      <c r="AM4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
@@ -2220,34 +2240,35 @@
       <c r="Z5" s="5"/>
       <c r="AA5" s="5"/>
       <c r="AB5" s="5"/>
-      <c r="AC5" s="7"/>
+      <c r="AC5" s="5"/>
       <c r="AD5" s="7"/>
-      <c r="AE5" s="11" t="str">
-        <f aca="false">IF(OR($A5="",$I5="",$AC5=""),"",$I5-$AC5-N($AD5))</f>
-        <v/>
-      </c>
-      <c r="AF5" s="12" t="str">
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="11" t="str">
+        <f aca="false">IF(OR($A5="",$I5="",$AD5=""),"",$I5-$AD5-N($AE5))</f>
+        <v/>
+      </c>
+      <c r="AG5" s="12" t="str">
         <f aca="false">IF($A5="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A5,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG5" s="13" t="str">
+      <c r="AH5" s="13" t="str">
         <f aca="false">IF($A5="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A5)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A5,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH5" s="11" t="str">
-        <f aca="false">IF($A5="","",IFERROR($AE5/$AG5,""))</f>
-        <v/>
-      </c>
-      <c r="AI5" s="13" t="str">
+      <c r="AI5" s="11" t="str">
+        <f aca="false">IF($A5="","",IFERROR($AF5/$AH5,""))</f>
+        <v/>
+      </c>
+      <c r="AJ5" s="13" t="str">
         <f aca="false">IF($A5="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A5,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ5" s="9" t="str">
+      <c r="AK5" s="9" t="str">
         <f aca="false">IF($A5="","",COUNTIFS(פניות!$B$2:$B$500,$A5,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK5" s="5"/>
       <c r="AL5" s="5"/>
+      <c r="AM5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
@@ -2299,34 +2320,35 @@
       <c r="Z6" s="5"/>
       <c r="AA6" s="5"/>
       <c r="AB6" s="5"/>
-      <c r="AC6" s="7"/>
+      <c r="AC6" s="5"/>
       <c r="AD6" s="7"/>
-      <c r="AE6" s="11" t="str">
-        <f aca="false">IF(OR($A6="",$I6="",$AC6=""),"",$I6-$AC6-N($AD6))</f>
-        <v/>
-      </c>
-      <c r="AF6" s="12" t="str">
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="11" t="str">
+        <f aca="false">IF(OR($A6="",$I6="",$AD6=""),"",$I6-$AD6-N($AE6))</f>
+        <v/>
+      </c>
+      <c r="AG6" s="12" t="str">
         <f aca="false">IF($A6="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A6,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG6" s="13" t="str">
+      <c r="AH6" s="13" t="str">
         <f aca="false">IF($A6="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A6)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A6,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH6" s="11" t="str">
-        <f aca="false">IF($A6="","",IFERROR($AE6/$AG6,""))</f>
-        <v/>
-      </c>
-      <c r="AI6" s="13" t="str">
+      <c r="AI6" s="11" t="str">
+        <f aca="false">IF($A6="","",IFERROR($AF6/$AH6,""))</f>
+        <v/>
+      </c>
+      <c r="AJ6" s="13" t="str">
         <f aca="false">IF($A6="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A6,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ6" s="9" t="str">
+      <c r="AK6" s="9" t="str">
         <f aca="false">IF($A6="","",COUNTIFS(פניות!$B$2:$B$500,$A6,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK6" s="5"/>
       <c r="AL6" s="5"/>
+      <c r="AM6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
@@ -2378,34 +2400,35 @@
       <c r="Z7" s="5"/>
       <c r="AA7" s="5"/>
       <c r="AB7" s="5"/>
-      <c r="AC7" s="7"/>
+      <c r="AC7" s="5"/>
       <c r="AD7" s="7"/>
-      <c r="AE7" s="11" t="str">
-        <f aca="false">IF(OR($A7="",$I7="",$AC7=""),"",$I7-$AC7-N($AD7))</f>
-        <v/>
-      </c>
-      <c r="AF7" s="12" t="str">
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="11" t="str">
+        <f aca="false">IF(OR($A7="",$I7="",$AD7=""),"",$I7-$AD7-N($AE7))</f>
+        <v/>
+      </c>
+      <c r="AG7" s="12" t="str">
         <f aca="false">IF($A7="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A7,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG7" s="13" t="str">
+      <c r="AH7" s="13" t="str">
         <f aca="false">IF($A7="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A7)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A7,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH7" s="11" t="str">
-        <f aca="false">IF($A7="","",IFERROR($AE7/$AG7,""))</f>
-        <v/>
-      </c>
-      <c r="AI7" s="13" t="str">
+      <c r="AI7" s="11" t="str">
+        <f aca="false">IF($A7="","",IFERROR($AF7/$AH7,""))</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="13" t="str">
         <f aca="false">IF($A7="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A7,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ7" s="9" t="str">
+      <c r="AK7" s="9" t="str">
         <f aca="false">IF($A7="","",COUNTIFS(פניות!$B$2:$B$500,$A7,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK7" s="5"/>
       <c r="AL7" s="5"/>
+      <c r="AM7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
@@ -2457,34 +2480,35 @@
       <c r="Z8" s="5"/>
       <c r="AA8" s="5"/>
       <c r="AB8" s="5"/>
-      <c r="AC8" s="7"/>
+      <c r="AC8" s="5"/>
       <c r="AD8" s="7"/>
-      <c r="AE8" s="11" t="str">
-        <f aca="false">IF(OR($A8="",$I8="",$AC8=""),"",$I8-$AC8-N($AD8))</f>
-        <v/>
-      </c>
-      <c r="AF8" s="12" t="str">
+      <c r="AE8" s="7"/>
+      <c r="AF8" s="11" t="str">
+        <f aca="false">IF(OR($A8="",$I8="",$AD8=""),"",$I8-$AD8-N($AE8))</f>
+        <v/>
+      </c>
+      <c r="AG8" s="12" t="str">
         <f aca="false">IF($A8="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A8,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG8" s="13" t="str">
+      <c r="AH8" s="13" t="str">
         <f aca="false">IF($A8="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A8)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A8,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH8" s="11" t="str">
-        <f aca="false">IF($A8="","",IFERROR($AE8/$AG8,""))</f>
-        <v/>
-      </c>
-      <c r="AI8" s="13" t="str">
+      <c r="AI8" s="11" t="str">
+        <f aca="false">IF($A8="","",IFERROR($AF8/$AH8,""))</f>
+        <v/>
+      </c>
+      <c r="AJ8" s="13" t="str">
         <f aca="false">IF($A8="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A8,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ8" s="9" t="str">
+      <c r="AK8" s="9" t="str">
         <f aca="false">IF($A8="","",COUNTIFS(פניות!$B$2:$B$500,$A8,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK8" s="5"/>
       <c r="AL8" s="5"/>
+      <c r="AM8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
@@ -2536,34 +2560,35 @@
       <c r="Z9" s="5"/>
       <c r="AA9" s="5"/>
       <c r="AB9" s="5"/>
-      <c r="AC9" s="7"/>
+      <c r="AC9" s="5"/>
       <c r="AD9" s="7"/>
-      <c r="AE9" s="11" t="str">
-        <f aca="false">IF(OR($A9="",$I9="",$AC9=""),"",$I9-$AC9-N($AD9))</f>
-        <v/>
-      </c>
-      <c r="AF9" s="12" t="str">
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="11" t="str">
+        <f aca="false">IF(OR($A9="",$I9="",$AD9=""),"",$I9-$AD9-N($AE9))</f>
+        <v/>
+      </c>
+      <c r="AG9" s="12" t="str">
         <f aca="false">IF($A9="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A9,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG9" s="13" t="str">
+      <c r="AH9" s="13" t="str">
         <f aca="false">IF($A9="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A9)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A9,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH9" s="11" t="str">
-        <f aca="false">IF($A9="","",IFERROR($AE9/$AG9,""))</f>
-        <v/>
-      </c>
-      <c r="AI9" s="13" t="str">
+      <c r="AI9" s="11" t="str">
+        <f aca="false">IF($A9="","",IFERROR($AF9/$AH9,""))</f>
+        <v/>
+      </c>
+      <c r="AJ9" s="13" t="str">
         <f aca="false">IF($A9="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A9,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ9" s="9" t="str">
+      <c r="AK9" s="9" t="str">
         <f aca="false">IF($A9="","",COUNTIFS(פניות!$B$2:$B$500,$A9,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK9" s="5"/>
       <c r="AL9" s="5"/>
+      <c r="AM9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
@@ -2615,34 +2640,35 @@
       <c r="Z10" s="5"/>
       <c r="AA10" s="5"/>
       <c r="AB10" s="5"/>
-      <c r="AC10" s="7"/>
+      <c r="AC10" s="5"/>
       <c r="AD10" s="7"/>
-      <c r="AE10" s="11" t="str">
-        <f aca="false">IF(OR($A10="",$I10="",$AC10=""),"",$I10-$AC10-N($AD10))</f>
-        <v/>
-      </c>
-      <c r="AF10" s="12" t="str">
+      <c r="AE10" s="7"/>
+      <c r="AF10" s="11" t="str">
+        <f aca="false">IF(OR($A10="",$I10="",$AD10=""),"",$I10-$AD10-N($AE10))</f>
+        <v/>
+      </c>
+      <c r="AG10" s="12" t="str">
         <f aca="false">IF($A10="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A10,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG10" s="13" t="str">
+      <c r="AH10" s="13" t="str">
         <f aca="false">IF($A10="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A10)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A10,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH10" s="11" t="str">
-        <f aca="false">IF($A10="","",IFERROR($AE10/$AG10,""))</f>
-        <v/>
-      </c>
-      <c r="AI10" s="13" t="str">
+      <c r="AI10" s="11" t="str">
+        <f aca="false">IF($A10="","",IFERROR($AF10/$AH10,""))</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="13" t="str">
         <f aca="false">IF($A10="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A10,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ10" s="9" t="str">
+      <c r="AK10" s="9" t="str">
         <f aca="false">IF($A10="","",COUNTIFS(פניות!$B$2:$B$500,$A10,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK10" s="5"/>
       <c r="AL10" s="5"/>
+      <c r="AM10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
@@ -2694,34 +2720,35 @@
       <c r="Z11" s="5"/>
       <c r="AA11" s="5"/>
       <c r="AB11" s="5"/>
-      <c r="AC11" s="7"/>
+      <c r="AC11" s="5"/>
       <c r="AD11" s="7"/>
-      <c r="AE11" s="11" t="str">
-        <f aca="false">IF(OR($A11="",$I11="",$AC11=""),"",$I11-$AC11-N($AD11))</f>
-        <v/>
-      </c>
-      <c r="AF11" s="12" t="str">
+      <c r="AE11" s="7"/>
+      <c r="AF11" s="11" t="str">
+        <f aca="false">IF(OR($A11="",$I11="",$AD11=""),"",$I11-$AD11-N($AE11))</f>
+        <v/>
+      </c>
+      <c r="AG11" s="12" t="str">
         <f aca="false">IF($A11="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A11,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG11" s="13" t="str">
+      <c r="AH11" s="13" t="str">
         <f aca="false">IF($A11="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A11)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A11,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH11" s="11" t="str">
-        <f aca="false">IF($A11="","",IFERROR($AE11/$AG11,""))</f>
-        <v/>
-      </c>
-      <c r="AI11" s="13" t="str">
+      <c r="AI11" s="11" t="str">
+        <f aca="false">IF($A11="","",IFERROR($AF11/$AH11,""))</f>
+        <v/>
+      </c>
+      <c r="AJ11" s="13" t="str">
         <f aca="false">IF($A11="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A11,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ11" s="9" t="str">
+      <c r="AK11" s="9" t="str">
         <f aca="false">IF($A11="","",COUNTIFS(פניות!$B$2:$B$500,$A11,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK11" s="5"/>
       <c r="AL11" s="5"/>
+      <c r="AM11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
@@ -2773,34 +2800,35 @@
       <c r="Z12" s="5"/>
       <c r="AA12" s="5"/>
       <c r="AB12" s="5"/>
-      <c r="AC12" s="7"/>
+      <c r="AC12" s="5"/>
       <c r="AD12" s="7"/>
-      <c r="AE12" s="11" t="str">
-        <f aca="false">IF(OR($A12="",$I12="",$AC12=""),"",$I12-$AC12-N($AD12))</f>
-        <v/>
-      </c>
-      <c r="AF12" s="12" t="str">
+      <c r="AE12" s="7"/>
+      <c r="AF12" s="11" t="str">
+        <f aca="false">IF(OR($A12="",$I12="",$AD12=""),"",$I12-$AD12-N($AE12))</f>
+        <v/>
+      </c>
+      <c r="AG12" s="12" t="str">
         <f aca="false">IF($A12="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A12,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG12" s="13" t="str">
+      <c r="AH12" s="13" t="str">
         <f aca="false">IF($A12="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A12)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A12,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH12" s="11" t="str">
-        <f aca="false">IF($A12="","",IFERROR($AE12/$AG12,""))</f>
-        <v/>
-      </c>
-      <c r="AI12" s="13" t="str">
+      <c r="AI12" s="11" t="str">
+        <f aca="false">IF($A12="","",IFERROR($AF12/$AH12,""))</f>
+        <v/>
+      </c>
+      <c r="AJ12" s="13" t="str">
         <f aca="false">IF($A12="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A12,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ12" s="9" t="str">
+      <c r="AK12" s="9" t="str">
         <f aca="false">IF($A12="","",COUNTIFS(פניות!$B$2:$B$500,$A12,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK12" s="5"/>
       <c r="AL12" s="5"/>
+      <c r="AM12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
@@ -2852,34 +2880,35 @@
       <c r="Z13" s="5"/>
       <c r="AA13" s="5"/>
       <c r="AB13" s="5"/>
-      <c r="AC13" s="7"/>
+      <c r="AC13" s="5"/>
       <c r="AD13" s="7"/>
-      <c r="AE13" s="11" t="str">
-        <f aca="false">IF(OR($A13="",$I13="",$AC13=""),"",$I13-$AC13-N($AD13))</f>
-        <v/>
-      </c>
-      <c r="AF13" s="12" t="str">
+      <c r="AE13" s="7"/>
+      <c r="AF13" s="11" t="str">
+        <f aca="false">IF(OR($A13="",$I13="",$AD13=""),"",$I13-$AD13-N($AE13))</f>
+        <v/>
+      </c>
+      <c r="AG13" s="12" t="str">
         <f aca="false">IF($A13="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A13,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG13" s="13" t="str">
+      <c r="AH13" s="13" t="str">
         <f aca="false">IF($A13="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A13)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A13,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH13" s="11" t="str">
-        <f aca="false">IF($A13="","",IFERROR($AE13/$AG13,""))</f>
-        <v/>
-      </c>
-      <c r="AI13" s="13" t="str">
+      <c r="AI13" s="11" t="str">
+        <f aca="false">IF($A13="","",IFERROR($AF13/$AH13,""))</f>
+        <v/>
+      </c>
+      <c r="AJ13" s="13" t="str">
         <f aca="false">IF($A13="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A13,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ13" s="9" t="str">
+      <c r="AK13" s="9" t="str">
         <f aca="false">IF($A13="","",COUNTIFS(פניות!$B$2:$B$500,$A13,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK13" s="5"/>
       <c r="AL13" s="5"/>
+      <c r="AM13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
@@ -2931,34 +2960,35 @@
       <c r="Z14" s="5"/>
       <c r="AA14" s="5"/>
       <c r="AB14" s="5"/>
-      <c r="AC14" s="7"/>
+      <c r="AC14" s="5"/>
       <c r="AD14" s="7"/>
-      <c r="AE14" s="11" t="str">
-        <f aca="false">IF(OR($A14="",$I14="",$AC14=""),"",$I14-$AC14-N($AD14))</f>
-        <v/>
-      </c>
-      <c r="AF14" s="12" t="str">
+      <c r="AE14" s="7"/>
+      <c r="AF14" s="11" t="str">
+        <f aca="false">IF(OR($A14="",$I14="",$AD14=""),"",$I14-$AD14-N($AE14))</f>
+        <v/>
+      </c>
+      <c r="AG14" s="12" t="str">
         <f aca="false">IF($A14="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A14,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG14" s="13" t="str">
+      <c r="AH14" s="13" t="str">
         <f aca="false">IF($A14="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A14)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A14,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH14" s="11" t="str">
-        <f aca="false">IF($A14="","",IFERROR($AE14/$AG14,""))</f>
-        <v/>
-      </c>
-      <c r="AI14" s="13" t="str">
+      <c r="AI14" s="11" t="str">
+        <f aca="false">IF($A14="","",IFERROR($AF14/$AH14,""))</f>
+        <v/>
+      </c>
+      <c r="AJ14" s="13" t="str">
         <f aca="false">IF($A14="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A14,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ14" s="9" t="str">
+      <c r="AK14" s="9" t="str">
         <f aca="false">IF($A14="","",COUNTIFS(פניות!$B$2:$B$500,$A14,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK14" s="5"/>
       <c r="AL14" s="5"/>
+      <c r="AM14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
@@ -3010,34 +3040,35 @@
       <c r="Z15" s="5"/>
       <c r="AA15" s="5"/>
       <c r="AB15" s="5"/>
-      <c r="AC15" s="7"/>
+      <c r="AC15" s="5"/>
       <c r="AD15" s="7"/>
-      <c r="AE15" s="11" t="str">
-        <f aca="false">IF(OR($A15="",$I15="",$AC15=""),"",$I15-$AC15-N($AD15))</f>
-        <v/>
-      </c>
-      <c r="AF15" s="12" t="str">
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="11" t="str">
+        <f aca="false">IF(OR($A15="",$I15="",$AD15=""),"",$I15-$AD15-N($AE15))</f>
+        <v/>
+      </c>
+      <c r="AG15" s="12" t="str">
         <f aca="false">IF($A15="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A15,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG15" s="13" t="str">
+      <c r="AH15" s="13" t="str">
         <f aca="false">IF($A15="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A15)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A15,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH15" s="11" t="str">
-        <f aca="false">IF($A15="","",IFERROR($AE15/$AG15,""))</f>
-        <v/>
-      </c>
-      <c r="AI15" s="13" t="str">
+      <c r="AI15" s="11" t="str">
+        <f aca="false">IF($A15="","",IFERROR($AF15/$AH15,""))</f>
+        <v/>
+      </c>
+      <c r="AJ15" s="13" t="str">
         <f aca="false">IF($A15="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A15,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ15" s="9" t="str">
+      <c r="AK15" s="9" t="str">
         <f aca="false">IF($A15="","",COUNTIFS(פניות!$B$2:$B$500,$A15,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK15" s="5"/>
       <c r="AL15" s="5"/>
+      <c r="AM15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
@@ -3089,34 +3120,35 @@
       <c r="Z16" s="5"/>
       <c r="AA16" s="5"/>
       <c r="AB16" s="5"/>
-      <c r="AC16" s="7"/>
+      <c r="AC16" s="5"/>
       <c r="AD16" s="7"/>
-      <c r="AE16" s="11" t="str">
-        <f aca="false">IF(OR($A16="",$I16="",$AC16=""),"",$I16-$AC16-N($AD16))</f>
-        <v/>
-      </c>
-      <c r="AF16" s="12" t="str">
+      <c r="AE16" s="7"/>
+      <c r="AF16" s="11" t="str">
+        <f aca="false">IF(OR($A16="",$I16="",$AD16=""),"",$I16-$AD16-N($AE16))</f>
+        <v/>
+      </c>
+      <c r="AG16" s="12" t="str">
         <f aca="false">IF($A16="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A16,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG16" s="13" t="str">
+      <c r="AH16" s="13" t="str">
         <f aca="false">IF($A16="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A16)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A16,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH16" s="11" t="str">
-        <f aca="false">IF($A16="","",IFERROR($AE16/$AG16,""))</f>
-        <v/>
-      </c>
-      <c r="AI16" s="13" t="str">
+      <c r="AI16" s="11" t="str">
+        <f aca="false">IF($A16="","",IFERROR($AF16/$AH16,""))</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="13" t="str">
         <f aca="false">IF($A16="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A16,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ16" s="9" t="str">
+      <c r="AK16" s="9" t="str">
         <f aca="false">IF($A16="","",COUNTIFS(פניות!$B$2:$B$500,$A16,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK16" s="5"/>
       <c r="AL16" s="5"/>
+      <c r="AM16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
@@ -3168,34 +3200,35 @@
       <c r="Z17" s="5"/>
       <c r="AA17" s="5"/>
       <c r="AB17" s="5"/>
-      <c r="AC17" s="7"/>
+      <c r="AC17" s="5"/>
       <c r="AD17" s="7"/>
-      <c r="AE17" s="11" t="str">
-        <f aca="false">IF(OR($A17="",$I17="",$AC17=""),"",$I17-$AC17-N($AD17))</f>
-        <v/>
-      </c>
-      <c r="AF17" s="12" t="str">
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="11" t="str">
+        <f aca="false">IF(OR($A17="",$I17="",$AD17=""),"",$I17-$AD17-N($AE17))</f>
+        <v/>
+      </c>
+      <c r="AG17" s="12" t="str">
         <f aca="false">IF($A17="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A17,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG17" s="13" t="str">
+      <c r="AH17" s="13" t="str">
         <f aca="false">IF($A17="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A17)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A17,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH17" s="11" t="str">
-        <f aca="false">IF($A17="","",IFERROR($AE17/$AG17,""))</f>
-        <v/>
-      </c>
-      <c r="AI17" s="13" t="str">
+      <c r="AI17" s="11" t="str">
+        <f aca="false">IF($A17="","",IFERROR($AF17/$AH17,""))</f>
+        <v/>
+      </c>
+      <c r="AJ17" s="13" t="str">
         <f aca="false">IF($A17="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A17,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ17" s="9" t="str">
+      <c r="AK17" s="9" t="str">
         <f aca="false">IF($A17="","",COUNTIFS(פניות!$B$2:$B$500,$A17,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK17" s="5"/>
       <c r="AL17" s="5"/>
+      <c r="AM17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
@@ -3247,34 +3280,35 @@
       <c r="Z18" s="5"/>
       <c r="AA18" s="5"/>
       <c r="AB18" s="5"/>
-      <c r="AC18" s="7"/>
+      <c r="AC18" s="5"/>
       <c r="AD18" s="7"/>
-      <c r="AE18" s="11" t="str">
-        <f aca="false">IF(OR($A18="",$I18="",$AC18=""),"",$I18-$AC18-N($AD18))</f>
-        <v/>
-      </c>
-      <c r="AF18" s="12" t="str">
+      <c r="AE18" s="7"/>
+      <c r="AF18" s="11" t="str">
+        <f aca="false">IF(OR($A18="",$I18="",$AD18=""),"",$I18-$AD18-N($AE18))</f>
+        <v/>
+      </c>
+      <c r="AG18" s="12" t="str">
         <f aca="false">IF($A18="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A18,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG18" s="13" t="str">
+      <c r="AH18" s="13" t="str">
         <f aca="false">IF($A18="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A18)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A18,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH18" s="11" t="str">
-        <f aca="false">IF($A18="","",IFERROR($AE18/$AG18,""))</f>
-        <v/>
-      </c>
-      <c r="AI18" s="13" t="str">
+      <c r="AI18" s="11" t="str">
+        <f aca="false">IF($A18="","",IFERROR($AF18/$AH18,""))</f>
+        <v/>
+      </c>
+      <c r="AJ18" s="13" t="str">
         <f aca="false">IF($A18="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A18,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ18" s="9" t="str">
+      <c r="AK18" s="9" t="str">
         <f aca="false">IF($A18="","",COUNTIFS(פניות!$B$2:$B$500,$A18,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK18" s="5"/>
       <c r="AL18" s="5"/>
+      <c r="AM18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
@@ -3326,34 +3360,35 @@
       <c r="Z19" s="5"/>
       <c r="AA19" s="5"/>
       <c r="AB19" s="5"/>
-      <c r="AC19" s="7"/>
+      <c r="AC19" s="5"/>
       <c r="AD19" s="7"/>
-      <c r="AE19" s="11" t="str">
-        <f aca="false">IF(OR($A19="",$I19="",$AC19=""),"",$I19-$AC19-N($AD19))</f>
-        <v/>
-      </c>
-      <c r="AF19" s="12" t="str">
+      <c r="AE19" s="7"/>
+      <c r="AF19" s="11" t="str">
+        <f aca="false">IF(OR($A19="",$I19="",$AD19=""),"",$I19-$AD19-N($AE19))</f>
+        <v/>
+      </c>
+      <c r="AG19" s="12" t="str">
         <f aca="false">IF($A19="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A19,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG19" s="13" t="str">
+      <c r="AH19" s="13" t="str">
         <f aca="false">IF($A19="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A19)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A19,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH19" s="11" t="str">
-        <f aca="false">IF($A19="","",IFERROR($AE19/$AG19,""))</f>
-        <v/>
-      </c>
-      <c r="AI19" s="13" t="str">
+      <c r="AI19" s="11" t="str">
+        <f aca="false">IF($A19="","",IFERROR($AF19/$AH19,""))</f>
+        <v/>
+      </c>
+      <c r="AJ19" s="13" t="str">
         <f aca="false">IF($A19="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A19,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ19" s="9" t="str">
+      <c r="AK19" s="9" t="str">
         <f aca="false">IF($A19="","",COUNTIFS(פניות!$B$2:$B$500,$A19,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK19" s="5"/>
       <c r="AL19" s="5"/>
+      <c r="AM19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
@@ -3405,34 +3440,35 @@
       <c r="Z20" s="5"/>
       <c r="AA20" s="5"/>
       <c r="AB20" s="5"/>
-      <c r="AC20" s="7"/>
+      <c r="AC20" s="5"/>
       <c r="AD20" s="7"/>
-      <c r="AE20" s="11" t="str">
-        <f aca="false">IF(OR($A20="",$I20="",$AC20=""),"",$I20-$AC20-N($AD20))</f>
-        <v/>
-      </c>
-      <c r="AF20" s="12" t="str">
+      <c r="AE20" s="7"/>
+      <c r="AF20" s="11" t="str">
+        <f aca="false">IF(OR($A20="",$I20="",$AD20=""),"",$I20-$AD20-N($AE20))</f>
+        <v/>
+      </c>
+      <c r="AG20" s="12" t="str">
         <f aca="false">IF($A20="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A20,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG20" s="13" t="str">
+      <c r="AH20" s="13" t="str">
         <f aca="false">IF($A20="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A20)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A20,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH20" s="11" t="str">
-        <f aca="false">IF($A20="","",IFERROR($AE20/$AG20,""))</f>
-        <v/>
-      </c>
-      <c r="AI20" s="13" t="str">
+      <c r="AI20" s="11" t="str">
+        <f aca="false">IF($A20="","",IFERROR($AF20/$AH20,""))</f>
+        <v/>
+      </c>
+      <c r="AJ20" s="13" t="str">
         <f aca="false">IF($A20="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A20,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ20" s="9" t="str">
+      <c r="AK20" s="9" t="str">
         <f aca="false">IF($A20="","",COUNTIFS(פניות!$B$2:$B$500,$A20,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK20" s="5"/>
       <c r="AL20" s="5"/>
+      <c r="AM20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
@@ -3484,34 +3520,35 @@
       <c r="Z21" s="5"/>
       <c r="AA21" s="5"/>
       <c r="AB21" s="5"/>
-      <c r="AC21" s="7"/>
+      <c r="AC21" s="5"/>
       <c r="AD21" s="7"/>
-      <c r="AE21" s="11" t="str">
-        <f aca="false">IF(OR($A21="",$I21="",$AC21=""),"",$I21-$AC21-N($AD21))</f>
-        <v/>
-      </c>
-      <c r="AF21" s="12" t="str">
+      <c r="AE21" s="7"/>
+      <c r="AF21" s="11" t="str">
+        <f aca="false">IF(OR($A21="",$I21="",$AD21=""),"",$I21-$AD21-N($AE21))</f>
+        <v/>
+      </c>
+      <c r="AG21" s="12" t="str">
         <f aca="false">IF($A21="","",IFERROR(INDEX(Checklist!$C$30:$G$30,MATCH($A21,Checklist!$C$1:$G$1,0)),""))</f>
         <v/>
       </c>
-      <c r="AG21" s="13" t="str">
+      <c r="AH21" s="13" t="str">
         <f aca="false">IF($A21="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A21)-SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A21,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AH21" s="11" t="str">
-        <f aca="false">IF($A21="","",IFERROR($AE21/$AG21,""))</f>
-        <v/>
-      </c>
-      <c r="AI21" s="13" t="str">
+      <c r="AI21" s="11" t="str">
+        <f aca="false">IF($A21="","",IFERROR($AF21/$AH21,""))</f>
+        <v/>
+      </c>
+      <c r="AJ21" s="13" t="str">
         <f aca="false">IF($A21="","",SUMIFS(שעות!$D$2:$D$500,שעות!$A$2:$A$500,$A21,שעות!$B$2:$B$500,"תמיכה (ריטיינר)"))</f>
         <v/>
       </c>
-      <c r="AJ21" s="9" t="str">
+      <c r="AK21" s="9" t="str">
         <f aca="false">IF($A21="","",COUNTIFS(פניות!$B$2:$B$500,$A21,פניות!$F$2:$F$500,"פתוחה"))</f>
         <v/>
       </c>
-      <c r="AK21" s="5"/>
       <c r="AL21" s="5"/>
+      <c r="AM21" s="5"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -3523,11 +3560,11 @@
       <formula1>"ליד,סקר בית,הצעה נשלחה,הזמנת ציוד,התקנה,בדיקות קבלה,פעיל,מושהה,הופסק"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="W2:W21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="X2:X21" type="list">
       <formula1>"כן,לא"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AA2:AA21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="AB2:AB21" type="list">
       <formula1>"כן,לא"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3558,10 +3595,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="4" t="str">
         <f aca="false">IF(לקוחות!$A2="","",לקוחות!$A2)</f>
@@ -3586,13 +3623,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="16"/>
@@ -3601,13 +3638,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
@@ -3616,13 +3653,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B4" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>79</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>77</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -3631,13 +3668,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -3646,13 +3683,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -3661,13 +3698,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -3676,13 +3713,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
@@ -3691,13 +3728,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -3706,13 +3743,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B10" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>87</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>85</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
@@ -3721,13 +3758,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
@@ -3736,13 +3773,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
@@ -3751,13 +3788,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
@@ -3766,13 +3803,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -3781,13 +3818,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
@@ -3796,13 +3833,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -3811,13 +3848,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
@@ -3826,13 +3863,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
@@ -3841,13 +3878,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
@@ -3856,13 +3893,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -3871,13 +3908,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
@@ -3886,13 +3923,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
@@ -3901,13 +3938,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
@@ -3916,13 +3953,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
@@ -3931,13 +3968,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
@@ -3946,13 +3983,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
@@ -3961,13 +3998,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
@@ -3976,13 +4013,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
@@ -3991,13 +4028,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -4007,7 +4044,7 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17"/>
       <c r="B30" s="18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C30" s="19" t="n">
         <f aca="false">IF(C$1="","",COUNTIF(C2:C29,"✓")/MAX(1,ROWS(C2:C29)-COUNTIF(C2:C29,"לא רלוונטי")))</f>
@@ -4075,30 +4112,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>46293</v>
@@ -4107,15 +4144,15 @@
         <v>1.5</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>46293</v>
@@ -4127,10 +4164,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>46300</v>
@@ -4142,10 +4179,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>46300</v>
@@ -4157,10 +4194,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>46303</v>
@@ -4169,15 +4206,15 @@
         <v>1.5</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>46309</v>
@@ -4186,15 +4223,15 @@
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>46314</v>
@@ -4206,10 +4243,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>46314</v>
@@ -4221,10 +4258,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>46314</v>
@@ -4236,10 +4273,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>46314</v>
@@ -4251,10 +4288,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>46316</v>
@@ -4263,15 +4300,15 @@
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>46328</v>
@@ -4280,7 +4317,7 @@
         <v>0.5</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4937,60 +4974,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" s="22" t="n">
         <v>46316.3819444445</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G2" s="22" t="n">
         <v>46316.4027777778</v>
@@ -5011,27 +5048,27 @@
         <v>✓</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="22" t="n">
         <v>46328.75</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G3" s="22"/>
       <c r="H3" s="22"/>
@@ -5048,7 +5085,7 @@
         <v/>
       </c>
       <c r="L3" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7350,21 +7387,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B2" s="25" t="n">
         <v>5700</v>
@@ -7378,7 +7415,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B3" s="25" t="n">
         <v>8700</v>
@@ -7389,7 +7426,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B4" s="25" t="n">
         <v>13150</v>
@@ -7400,17 +7437,17 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">COUNTIF(לקוחות!$S$2:$S$21,"פעיל")</f>
@@ -7419,7 +7456,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">SUMIFS(לקוחות!$G$2:$G$21,לקוחות!$S$2:$S$21,"פעיל")</f>
@@ -7428,7 +7465,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B11" s="29" t="n">
         <f aca="false">COUNTIF(פניות!$F$2:$F$500,"פתוחה")</f>
@@ -7437,7 +7474,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B12" s="29" t="n">
         <f aca="false">COUNTIFS(פניות!$E$2:$E$500,"קריטי",פניות!$K$2:$K$500,"✗")</f>
@@ -7446,7 +7483,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B13" s="31" t="n">
         <f aca="false">SUM(שעות!$D$2:$D$500)-SUMIFS(שעות!$D$2:$D$500,שעות!$B$2:$B$500,"תמיכה (ריטיינר)")</f>
@@ -7455,7 +7492,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B14" s="30" t="n">
         <f aca="false">SUM(לקוחות!$N$2:$N$21)</f>
@@ -7464,7 +7501,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B15" s="31" t="n">
         <f aca="false">SUMIFS(שעות!$D$2:$D$500,שעות!$B$2:$B$500,"תמיכה (ריטיינר)")</f>

</xml_diff>